<commit_message>
Add legal entity setup and part-time financist to Flyby budget
New one-time line: legal structure setup ($10,000). New payroll line:
part-time financist ($1,500/mo). Accountant was already budgeted.
New total: $652,080 for 6 months.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LctDpe2FhgqULyBDcZhWXD
</commit_message>
<xml_diff>
--- a/flyby-budget-6-months.xlsx
+++ b/flyby-budget-6-months.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="69">
   <si>
     <t xml:space="preserve">Проєкт Flyby — кошторис на 6 місяців</t>
   </si>
@@ -91,10 +91,16 @@
     <t xml:space="preserve">ДОДАНО: закупівля комплектуючих на 100 девайсів, логістика; оцінка з ринку</t>
   </si>
   <si>
+    <t xml:space="preserve">Фінансист (part-time)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Запит замовника: фінмодель, управлінський облік, звітність для інвесторів; ставка — оцінка з ринку (part-time)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Бухгалтер (аутсорс, part-time)</t>
   </si>
   <si>
-    <t xml:space="preserve">ДОДАНО: облік, зарплати, звітність; оцінка з ринку (аутсорс)</t>
+    <t xml:space="preserve">Запит замовника: облік, зарплати, звітність; ставка — оцінка з ринку (аутсорс)</t>
   </si>
   <si>
     <t xml:space="preserve">Разом ФОП</t>
@@ -163,6 +169,18 @@
     <t xml:space="preserve">Разом операційні</t>
   </si>
   <si>
+    <t xml:space="preserve">5. Разові витрати</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Створення юридичної структури</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Запит замовника. Реєстрація компанії (холдинг + операційна), статутні документи, IP-договори, банківські рахунки; оцінка. Разова витрата, у колонці 'міс' — усереднення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Разом разові</t>
+  </si>
+  <si>
     <t xml:space="preserve">ПІДСУМОК</t>
   </si>
   <si>
@@ -178,6 +196,9 @@
     <t xml:space="preserve">Операційні витрати</t>
   </si>
   <si>
+    <t xml:space="preserve">Разові витрати (юрструктура)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Проміжний підсумок</t>
   </si>
   <si>
@@ -190,10 +211,10 @@
     <t xml:space="preserve">РАЗОМ НА 6 МІСЯЦІВ</t>
   </si>
   <si>
-    <t xml:space="preserve">Середній burn rate на місяць (без разової закупівлі)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ФОП + виставки + опекс + резерв, без $200k комплектуючих</t>
+    <t xml:space="preserve">Середній burn rate на місяць (без разових витрат)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ФОП + виставки + опекс + резерв, без комплектуючих ($200k) та юрструктури ($10k)</t>
   </si>
   <si>
     <t xml:space="preserve">Легенда:</t>
@@ -746,7 +767,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
@@ -993,7 +1014,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
         <v>23</v>
       </c>
@@ -1001,154 +1022,154 @@
         <v>1</v>
       </c>
       <c r="C15" s="8" t="n">
-        <v>800</v>
+        <v>1500</v>
       </c>
       <c r="D15" s="9" t="n">
         <f aca="false">B15*C15</f>
-        <v>800</v>
+        <v>1500</v>
       </c>
       <c r="E15" s="9" t="n">
         <f aca="false">D15*6</f>
-        <v>4800</v>
+        <v>9000</v>
       </c>
       <c r="F15" s="10" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="13" t="n">
-        <f aca="false">SUM(D6:D15)</f>
-        <v>45800</v>
-      </c>
-      <c r="E16" s="13" t="n">
-        <f aca="false">SUM(E6:E15)</f>
-        <v>274800</v>
-      </c>
-      <c r="F16" s="12"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="B16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="8" t="n">
+        <v>800</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <f aca="false">B16*C16</f>
+        <v>800</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <f aca="false">D16*6</f>
+        <v>4800</v>
+      </c>
+      <c r="F16" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="13" t="n">
+        <f aca="false">SUM(D6:D16)</f>
+        <v>47300</v>
+      </c>
+      <c r="E17" s="13" t="n">
+        <f aca="false">SUM(E6:E16)</f>
+        <v>283800</v>
+      </c>
+      <c r="F17" s="12"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B20" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C20" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="D20" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E19" s="5" t="s">
+      <c r="E20" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F19" s="5" t="s">
+      <c r="F20" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B20" s="7" t="n">
+    <row r="21" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="C20" s="8" t="n">
+      <c r="C21" s="8" t="n">
         <v>2000</v>
       </c>
-      <c r="D20" s="9" t="n">
-        <f aca="false">E20/6</f>
+      <c r="D21" s="9" t="n">
+        <f aca="false">E21/6</f>
         <v>33333.3333333333</v>
       </c>
-      <c r="E20" s="9" t="n">
-        <f aca="false">B20*C20</f>
+      <c r="E21" s="9" t="n">
+        <f aca="false">B21*C21</f>
         <v>200000</v>
       </c>
-      <c r="F20" s="10" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="B21" s="12"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="13" t="n">
-        <f aca="false">SUM(D20:D20)</f>
+      <c r="F21" s="10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B22" s="12"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="13" t="n">
+        <f aca="false">SUM(D21:D21)</f>
         <v>33333.3333333333</v>
       </c>
-      <c r="E21" s="13" t="n">
-        <f aca="false">SUM(E20:E20)</f>
+      <c r="E22" s="13" t="n">
+        <f aca="false">SUM(E21:E21)</f>
         <v>200000</v>
       </c>
-      <c r="F21" s="12"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
+      <c r="F22" s="12"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B25" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C25" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D25" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E24" s="5" t="s">
+      <c r="E25" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F24" s="5" t="s">
+      <c r="F25" s="5" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B25" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C25" s="8" t="n">
-        <v>2500</v>
-      </c>
-      <c r="D25" s="9" t="n">
-        <f aca="false">B25*C25</f>
-        <v>2500</v>
-      </c>
-      <c r="E25" s="9" t="n">
-        <f aca="false">D25*6</f>
-        <v>15000</v>
-      </c>
-      <c r="F25" s="10" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1159,15 +1180,15 @@
         <v>1</v>
       </c>
       <c r="C26" s="8" t="n">
-        <v>3500</v>
+        <v>2500</v>
       </c>
       <c r="D26" s="9" t="n">
         <f aca="false">B26*C26</f>
-        <v>3500</v>
+        <v>2500</v>
       </c>
       <c r="E26" s="9" t="n">
         <f aca="false">D26*6</f>
-        <v>21000</v>
+        <v>15000</v>
       </c>
       <c r="F26" s="10" t="s">
         <v>34</v>
@@ -1181,86 +1202,86 @@
         <v>1</v>
       </c>
       <c r="C27" s="8" t="n">
-        <v>4500</v>
+        <v>3500</v>
       </c>
       <c r="D27" s="9" t="n">
         <f aca="false">B27*C27</f>
-        <v>4500</v>
+        <v>3500</v>
       </c>
       <c r="E27" s="9" t="n">
         <f aca="false">D27*6</f>
+        <v>21000</v>
+      </c>
+      <c r="F27" s="10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" s="8" t="n">
+        <v>4500</v>
+      </c>
+      <c r="D28" s="9" t="n">
+        <f aca="false">B28*C28</f>
+        <v>4500</v>
+      </c>
+      <c r="E28" s="9" t="n">
+        <f aca="false">D28*6</f>
         <v>27000</v>
       </c>
-      <c r="F27" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="11" t="s">
+      <c r="F28" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B28" s="12"/>
-      <c r="C28" s="12"/>
-      <c r="D28" s="13" t="n">
-        <f aca="false">SUM(D25:D27)</f>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B29" s="12"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="13" t="n">
+        <f aca="false">SUM(D26:D28)</f>
         <v>10500</v>
       </c>
-      <c r="E28" s="13" t="n">
-        <f aca="false">SUM(E25:E27)</f>
+      <c r="E29" s="13" t="n">
+        <f aca="false">SUM(E26:E28)</f>
         <v>63000</v>
       </c>
-      <c r="F28" s="12"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B30" s="4"/>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
+      <c r="F29" s="12"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="s">
+      <c r="A31" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="B32" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="C32" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D31" s="5" t="s">
+      <c r="D32" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E31" s="5" t="s">
+      <c r="E32" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F31" s="5" t="s">
+      <c r="F32" s="5" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B32" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" s="8" t="n">
-        <v>2000</v>
-      </c>
-      <c r="D32" s="9" t="n">
-        <f aca="false">B32*C32</f>
-        <v>2000</v>
-      </c>
-      <c r="E32" s="9" t="n">
-        <f aca="false">D32*6</f>
-        <v>12000</v>
-      </c>
-      <c r="F32" s="10" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1285,7 +1306,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
         <v>42</v>
       </c>
@@ -1293,21 +1314,21 @@
         <v>1</v>
       </c>
       <c r="C34" s="8" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="D34" s="9" t="n">
         <f aca="false">B34*C34</f>
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="E34" s="9" t="n">
         <f aca="false">D34*6</f>
-        <v>6000</v>
+        <v>12000</v>
       </c>
       <c r="F34" s="10" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
         <v>44</v>
       </c>
@@ -1330,177 +1351,283 @@
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="11" t="s">
+      <c r="A36" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B36" s="12"/>
-      <c r="C36" s="12"/>
-      <c r="D36" s="13" t="n">
-        <f aca="false">SUM(D32:D35)</f>
+      <c r="B36" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D36" s="9" t="n">
+        <f aca="false">B36*C36</f>
+        <v>1000</v>
+      </c>
+      <c r="E36" s="9" t="n">
+        <f aca="false">D36*6</f>
         <v>6000</v>
       </c>
-      <c r="E36" s="13" t="n">
-        <f aca="false">SUM(E32:E35)</f>
+      <c r="F36" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B37" s="12"/>
+      <c r="C37" s="12"/>
+      <c r="D37" s="13" t="n">
+        <f aca="false">SUM(D33:D36)</f>
+        <v>6000</v>
+      </c>
+      <c r="E37" s="13" t="n">
+        <f aca="false">SUM(E33:E36)</f>
         <v>36000</v>
       </c>
-      <c r="F36" s="12"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B38" s="4"/>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="4"/>
-      <c r="F38" s="4"/>
+      <c r="F37" s="12"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="B39" s="14"/>
-      <c r="C39" s="14"/>
-      <c r="D39" s="15" t="n">
-        <f aca="false">D16</f>
-        <v>45800</v>
-      </c>
-      <c r="E39" s="15" t="n">
-        <f aca="false">E16</f>
-        <v>274800</v>
-      </c>
-      <c r="F39" s="14"/>
+      <c r="A39" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B39" s="4"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="B40" s="14"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="15" t="n">
-        <f aca="false">D21</f>
-        <v>33333.3333333333</v>
-      </c>
-      <c r="E40" s="15" t="n">
-        <f aca="false">E21</f>
-        <v>200000</v>
-      </c>
-      <c r="F40" s="14"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="15" t="n">
-        <f aca="false">D28</f>
+      <c r="B41" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" s="8" t="n">
+        <v>10000</v>
+      </c>
+      <c r="D41" s="9" t="n">
+        <f aca="false">E41/6</f>
+        <v>1666.66666666667</v>
+      </c>
+      <c r="E41" s="9" t="n">
+        <f aca="false">B41*C41</f>
+        <v>10000</v>
+      </c>
+      <c r="F41" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B42" s="12"/>
+      <c r="C42" s="12"/>
+      <c r="D42" s="13" t="n">
+        <f aca="false">SUM(D41:D41)</f>
+        <v>1666.66666666667</v>
+      </c>
+      <c r="E42" s="13" t="n">
+        <f aca="false">SUM(E41:E41)</f>
+        <v>10000</v>
+      </c>
+      <c r="F42" s="12"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+      <c r="E44" s="4"/>
+      <c r="F44" s="4"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B45" s="14"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="15" t="n">
+        <f aca="false">D17</f>
+        <v>47300</v>
+      </c>
+      <c r="E45" s="15" t="n">
+        <f aca="false">E17</f>
+        <v>283800</v>
+      </c>
+      <c r="F45" s="14"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B46" s="14"/>
+      <c r="C46" s="14"/>
+      <c r="D46" s="15" t="n">
+        <f aca="false">D22</f>
+        <v>33333.3333333333</v>
+      </c>
+      <c r="E46" s="15" t="n">
+        <f aca="false">E22</f>
+        <v>200000</v>
+      </c>
+      <c r="F46" s="14"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B47" s="14"/>
+      <c r="C47" s="14"/>
+      <c r="D47" s="15" t="n">
+        <f aca="false">D29</f>
         <v>10500</v>
       </c>
-      <c r="E41" s="15" t="n">
-        <f aca="false">E28</f>
+      <c r="E47" s="15" t="n">
+        <f aca="false">E29</f>
         <v>63000</v>
       </c>
-      <c r="F41" s="14"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B42" s="14"/>
-      <c r="C42" s="14"/>
-      <c r="D42" s="15" t="n">
-        <f aca="false">D36</f>
+      <c r="F47" s="14"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B48" s="14"/>
+      <c r="C48" s="14"/>
+      <c r="D48" s="15" t="n">
+        <f aca="false">D37</f>
         <v>6000</v>
       </c>
-      <c r="E42" s="15" t="n">
-        <f aca="false">E36</f>
+      <c r="E48" s="15" t="n">
+        <f aca="false">E37</f>
         <v>36000</v>
       </c>
-      <c r="F42" s="14"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="B43" s="14"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="17" t="n">
-        <f aca="false">SUM(D39:D42)</f>
-        <v>95633.3333333333</v>
-      </c>
-      <c r="E43" s="17" t="n">
-        <f aca="false">SUM(E39:E42)</f>
-        <v>573800</v>
-      </c>
-      <c r="F43" s="14"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="B44" s="18" t="n">
+      <c r="F48" s="14"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B49" s="14"/>
+      <c r="C49" s="14"/>
+      <c r="D49" s="15" t="n">
+        <f aca="false">D42</f>
+        <v>1666.66666666667</v>
+      </c>
+      <c r="E49" s="15" t="n">
+        <f aca="false">E42</f>
+        <v>10000</v>
+      </c>
+      <c r="F49" s="14"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="B50" s="14"/>
+      <c r="C50" s="14"/>
+      <c r="D50" s="17" t="n">
+        <f aca="false">SUM(D45:D49)</f>
+        <v>98800</v>
+      </c>
+      <c r="E50" s="17" t="n">
+        <f aca="false">SUM(E45:E49)</f>
+        <v>592800</v>
+      </c>
+      <c r="F50" s="14"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B51" s="18" t="n">
         <v>0.1</v>
       </c>
-      <c r="C44" s="14"/>
-      <c r="D44" s="9" t="n">
-        <f aca="false">D43*B44</f>
-        <v>9563.33333333333</v>
-      </c>
-      <c r="E44" s="9" t="n">
-        <f aca="false">E43*B44</f>
-        <v>57380</v>
-      </c>
-      <c r="F44" s="19" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="20" t="s">
-        <v>55</v>
-      </c>
-      <c r="B45" s="21"/>
-      <c r="C45" s="21"/>
-      <c r="D45" s="22" t="n">
-        <f aca="false">D43+D44</f>
-        <v>105196.666666667</v>
-      </c>
-      <c r="E45" s="22" t="n">
-        <f aca="false">E43+E44</f>
-        <v>631180</v>
-      </c>
-      <c r="F45" s="21"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="D46" s="24" t="n">
-        <f aca="false">(E45-E21)/6</f>
-        <v>71863.3333333333</v>
-      </c>
-      <c r="F46" s="25" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="23" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="26" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="25" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="25" t="s">
+      <c r="C51" s="14"/>
+      <c r="D51" s="9" t="n">
+        <f aca="false">D50*B51</f>
+        <v>9880</v>
+      </c>
+      <c r="E51" s="9" t="n">
+        <f aca="false">E50*B51</f>
+        <v>59280</v>
+      </c>
+      <c r="F51" s="19" t="s">
         <v>61</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="20" t="s">
+        <v>62</v>
+      </c>
+      <c r="B52" s="21"/>
+      <c r="C52" s="21"/>
+      <c r="D52" s="22" t="n">
+        <f aca="false">D50+D51</f>
+        <v>108680</v>
+      </c>
+      <c r="E52" s="22" t="n">
+        <f aca="false">E50+E51</f>
+        <v>652080</v>
+      </c>
+      <c r="F52" s="21"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="D53" s="24" t="n">
+        <f aca="false">(E52-E22-E42)/6</f>
+        <v>73680</v>
+      </c>
+      <c r="F53" s="25" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="23" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="26" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="25" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="25" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>